<commit_message>
Correções no arquivo de estado dos processos foram feitas e grandes melhorias no frontend para visualização do estado dos processos por recebimento
</commit_message>
<xml_diff>
--- a/Estado_Processos_Recebimento.xlsx
+++ b/Estado_Processos_Recebimento.xlsx
@@ -562,36 +562,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>100001</t>
+          <t>100002</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>50</v>
+        <v>5000</v>
       </c>
       <c r="C2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="D2" t="n">
-        <v>20</v>
-      </c>
       <c r="E2" t="n">
-        <v>20</v>
-      </c>
-      <c r="F2" t="n">
-        <v>30</v>
-      </c>
+        <v>1000</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" t="n">
-        <v>0.06340000000000001</v>
-      </c>
       <c r="I2" t="n">
-        <v>0.06340000000000001</v>
+        <v>10</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>FATURADO</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -601,14 +599,10 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>CALCULADO</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>08/2025</t>
-        </is>
-      </c>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>{"Alessandro Cappi": 0.010000000000000002}</t>
@@ -616,17 +610,17 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 0.317}</t>
+          <t>{"Alessandro Cappi": 1.0}</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Detector Portátil", "subgrupo": "MicroClip", "tipo_mercadoria": "Produto", "valor": 50.0, "taxa": 0.010000000000000002, "fc": 0.317, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 70.0, "meta": 100.0, "atingimento": 0.7, "atingimento_cap": 0.7, "componente_fc": 0.105}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 20.0, "meta": 100.0, "atingimento": 0.2, "atingimento_cap": 0.2, "componente_fc": 0.06}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.38, "meta": 0.5, "atingimento": 0.76, "atingimento_cap": 0.76, "componente_fc": 0.15200000000000002}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 66.66666666666667, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.317}}], "total_valor": 50.0, "soma_ponderada": 0.5000000000000001, "tcmp_final": 0.010000000000000002}}</t>
+          <t>{"Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Detector Portátil", "subgrupo": "MicroClip", "tipo_mercadoria": "Produto", "valor": 5000.0, "taxa": 0.010000000000000002, "fc": 1.0, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": null}], "total_valor": 5000.0, "soma_ponderada": 50.00000000000001, "tcmp_final": 0.010000000000000002}}</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Detector Portátil", "subgrupo": "MicroClip", "tipo_mercadoria": "Produto", "valor": 50.0, "taxa": 0.010000000000000002, "fc": 0.317, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 70.0, "meta": 100.0, "atingimento": 0.7, "atingimento_cap": 0.7, "componente_fc": 0.105}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 20.0, "meta": 100.0, "atingimento": 0.2, "atingimento_cap": 0.2, "componente_fc": 0.06}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.38, "meta": 0.5, "atingimento": 0.76, "atingimento_cap": 0.76, "componente_fc": 0.15200000000000002}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 66.66666666666667, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.317}}], "total_valor": 50.0, "soma_ponderada": 15.85, "fcmp_final": 0.317}}</t>
+          <t>{"Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Detector Portátil", "subgrupo": "MicroClip", "tipo_mercadoria": "Produto", "valor": 5000.0, "taxa": 0.010000000000000002, "fc": 1.0, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": null}], "total_valor": 5000.0, "soma_ponderada": 5000.0, "fcmp_final": 1.0}}</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -635,20 +629,20 @@
         </is>
       </c>
       <c r="S2" s="2" t="n">
-        <v>45879</v>
+        <v>45870</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>45879</v>
+        <v>45870</v>
       </c>
       <c r="U2" t="n">
         <v>1</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>45995.63094627377</v>
+        <v>46000.5783992941</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{"Alessandro Cappi": 10.000000000000002}</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
Versão robô de comissões antes da exclusão dos testes antigos e criação de testes unitários e de integração totalmente novos e planejados
</commit_message>
<xml_diff>
--- a/Estado_Processos_Recebimento.xlsx
+++ b/Estado_Processos_Recebimento.xlsx
@@ -644,7 +644,7 @@
         <v>1</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>46070.97325991028</v>
+        <v>46072.61991042176</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -743,7 +743,7 @@
         <v>1</v>
       </c>
       <c r="V3" s="2" t="n">
-        <v>46070.97326020588</v>
+        <v>46072.61991158671</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>

</xml_diff>